<commit_message>
Add Risk Misc regime (remaining 50 titles) to the download plan
Relabel the 50 out-of-scope titles as the "Misc" regime and give them a
dedicated folder alongside Banking and Insurance. Misc covers general
op/conduct/resilience risk, buy-side/portfolio management, tech/AI & data,
energy & commodities, and ESG & climate.

fetch_riskbooks.py gains --regime misc, filing them under a "Risk Misc"
top-level folder (and matching Drive subfolder). Adds RiskBooks_misc.csv and
refreshes RiskBooks_download_plan.* with the regime column now covering all
three regimes (Banking 49, Insurance 8, Misc 50 = 107).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AGRjrE3Jo22ZAxhTiwwc9s
</commit_message>
<xml_diff>
--- a/riskbooks/RiskBooks_download_plan.xlsx
+++ b/riskbooks/RiskBooks_download_plan.xlsx
@@ -100,7 +100,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -572,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -667,7 +667,7 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Neither regime</t>
+          <t>Risk Misc</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
@@ -675,7 +675,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Energy, buy-side, ESG, tech, general op/conduct risk. Listed, not scheduled.</t>
+          <t>Everything outside both prudential regimes: op/conduct risk, buy-side, tech/AI, energy, ESG. Saved to its own folder.</t>
         </is>
       </c>
     </row>
@@ -702,10 +702,20 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
+          <t>Risk Misc total</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
           <t>All titles</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B13" s="9" t="n">
         <v>107</v>
       </c>
     </row>
@@ -3133,13 +3143,11 @@
     <row r="59">
       <c r="A59" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B59" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B59" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C59" s="27" t="inlineStr">
         <is>
@@ -3176,13 +3184,11 @@
     <row r="60">
       <c r="A60" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B60" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B60" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C60" s="27" t="inlineStr">
         <is>
@@ -3219,13 +3225,11 @@
     <row r="61">
       <c r="A61" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B61" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B61" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C61" s="27" t="inlineStr">
         <is>
@@ -3262,13 +3266,11 @@
     <row r="62">
       <c r="A62" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B62" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B62" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C62" s="27" t="inlineStr">
         <is>
@@ -3305,13 +3307,11 @@
     <row r="63">
       <c r="A63" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B63" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B63" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C63" s="27" t="inlineStr">
         <is>
@@ -3348,13 +3348,11 @@
     <row r="64">
       <c r="A64" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B64" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B64" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C64" s="27" t="inlineStr">
         <is>
@@ -3391,13 +3389,11 @@
     <row r="65">
       <c r="A65" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B65" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B65" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C65" s="27" t="inlineStr">
         <is>
@@ -3434,13 +3430,11 @@
     <row r="66">
       <c r="A66" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B66" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B66" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C66" s="27" t="inlineStr">
         <is>
@@ -3477,13 +3471,11 @@
     <row r="67">
       <c r="A67" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B67" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B67" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C67" s="27" t="inlineStr">
         <is>
@@ -3520,13 +3512,11 @@
     <row r="68">
       <c r="A68" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B68" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B68" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C68" s="27" t="inlineStr">
         <is>
@@ -3563,13 +3553,11 @@
     <row r="69">
       <c r="A69" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B69" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B69" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C69" s="27" t="inlineStr">
         <is>
@@ -3606,13 +3594,11 @@
     <row r="70">
       <c r="A70" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B70" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B70" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C70" s="27" t="inlineStr">
         <is>
@@ -3649,13 +3635,11 @@
     <row r="71">
       <c r="A71" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B71" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B71" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C71" s="27" t="inlineStr">
         <is>
@@ -3692,13 +3676,11 @@
     <row r="72">
       <c r="A72" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B72" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B72" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C72" s="27" t="inlineStr">
         <is>
@@ -3735,13 +3717,11 @@
     <row r="73">
       <c r="A73" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B73" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B73" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C73" s="27" t="inlineStr">
         <is>
@@ -3778,13 +3758,11 @@
     <row r="74">
       <c r="A74" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B74" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B74" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C74" s="27" t="inlineStr">
         <is>
@@ -3821,13 +3799,11 @@
     <row r="75">
       <c r="A75" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B75" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B75" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C75" s="27" t="inlineStr">
         <is>
@@ -3864,13 +3840,11 @@
     <row r="76">
       <c r="A76" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B76" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B76" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C76" s="27" t="inlineStr">
         <is>
@@ -3907,13 +3881,11 @@
     <row r="77">
       <c r="A77" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B77" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B77" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C77" s="27" t="inlineStr">
         <is>
@@ -3950,13 +3922,11 @@
     <row r="78">
       <c r="A78" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B78" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B78" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C78" s="27" t="inlineStr">
         <is>
@@ -3993,13 +3963,11 @@
     <row r="79">
       <c r="A79" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B79" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B79" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C79" s="27" t="inlineStr">
         <is>
@@ -4036,13 +4004,11 @@
     <row r="80">
       <c r="A80" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B80" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B80" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C80" s="27" t="inlineStr">
         <is>
@@ -4079,13 +4045,11 @@
     <row r="81">
       <c r="A81" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B81" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B81" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C81" s="27" t="inlineStr">
         <is>
@@ -4122,13 +4086,11 @@
     <row r="82">
       <c r="A82" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B82" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B82" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C82" s="27" t="inlineStr">
         <is>
@@ -4165,13 +4127,11 @@
     <row r="83">
       <c r="A83" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B83" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B83" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C83" s="27" t="inlineStr">
         <is>
@@ -4208,13 +4168,11 @@
     <row r="84">
       <c r="A84" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B84" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B84" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C84" s="27" t="inlineStr">
         <is>
@@ -4251,13 +4209,11 @@
     <row r="85">
       <c r="A85" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B85" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B85" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C85" s="27" t="inlineStr">
         <is>
@@ -4294,13 +4250,11 @@
     <row r="86">
       <c r="A86" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B86" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B86" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C86" s="27" t="inlineStr">
         <is>
@@ -4337,13 +4291,11 @@
     <row r="87">
       <c r="A87" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B87" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B87" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C87" s="27" t="inlineStr">
         <is>
@@ -4380,13 +4332,11 @@
     <row r="88">
       <c r="A88" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B88" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B88" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C88" s="27" t="inlineStr">
         <is>
@@ -4423,13 +4373,11 @@
     <row r="89">
       <c r="A89" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B89" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B89" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C89" s="27" t="inlineStr">
         <is>
@@ -4466,13 +4414,11 @@
     <row r="90">
       <c r="A90" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B90" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B90" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C90" s="27" t="inlineStr">
         <is>
@@ -4509,13 +4455,11 @@
     <row r="91">
       <c r="A91" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B91" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B91" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C91" s="27" t="inlineStr">
         <is>
@@ -4552,13 +4496,11 @@
     <row r="92">
       <c r="A92" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B92" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B92" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C92" s="27" t="inlineStr">
         <is>
@@ -4595,13 +4537,11 @@
     <row r="93">
       <c r="A93" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B93" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B93" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C93" s="27" t="inlineStr">
         <is>
@@ -4638,13 +4578,11 @@
     <row r="94">
       <c r="A94" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B94" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B94" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C94" s="27" t="inlineStr">
         <is>
@@ -4681,13 +4619,11 @@
     <row r="95">
       <c r="A95" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B95" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B95" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C95" s="27" t="inlineStr">
         <is>
@@ -4724,13 +4660,11 @@
     <row r="96">
       <c r="A96" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B96" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B96" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C96" s="27" t="inlineStr">
         <is>
@@ -4767,13 +4701,11 @@
     <row r="97">
       <c r="A97" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B97" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B97" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C97" s="27" t="inlineStr">
         <is>
@@ -4810,13 +4742,11 @@
     <row r="98">
       <c r="A98" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B98" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B98" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C98" s="27" t="inlineStr">
         <is>
@@ -4853,13 +4783,11 @@
     <row r="99">
       <c r="A99" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B99" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B99" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C99" s="27" t="inlineStr">
         <is>
@@ -4896,13 +4824,11 @@
     <row r="100">
       <c r="A100" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B100" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B100" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C100" s="27" t="inlineStr">
         <is>
@@ -4939,13 +4865,11 @@
     <row r="101">
       <c r="A101" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B101" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B101" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C101" s="27" t="inlineStr">
         <is>
@@ -4982,13 +4906,11 @@
     <row r="102">
       <c r="A102" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B102" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B102" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C102" s="27" t="inlineStr">
         <is>
@@ -5025,13 +4947,11 @@
     <row r="103">
       <c r="A103" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B103" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B103" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C103" s="27" t="inlineStr">
         <is>
@@ -5068,13 +4988,11 @@
     <row r="104">
       <c r="A104" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B104" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B104" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C104" s="27" t="inlineStr">
         <is>
@@ -5111,13 +5029,11 @@
     <row r="105">
       <c r="A105" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B105" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B105" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C105" s="27" t="inlineStr">
         <is>
@@ -5154,13 +5070,11 @@
     <row r="106">
       <c r="A106" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B106" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B106" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C106" s="27" t="inlineStr">
         <is>
@@ -5197,13 +5111,11 @@
     <row r="107">
       <c r="A107" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B107" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B107" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C107" s="27" t="inlineStr">
         <is>
@@ -5240,13 +5152,11 @@
     <row r="108">
       <c r="A108" s="27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B108" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="B108" s="27" t="n">
+        <v>1</v>
       </c>
       <c r="C108" s="27" t="inlineStr">
         <is>
@@ -5283,7 +5193,7 @@
     <row r="110">
       <c r="A110" s="31" t="inlineStr">
         <is>
-          <t>Two prudential regimes, filed separately. BANKING (49) in download waves: Wave 1 Tier-1 core (capital, derivatives, credit derivatives, counterparty/collateral); Wave 2 all remaining credit + regulatory (FRTB, stress testing, IFRS 9/CECL, model risk, systemic); Wave 3 rest of the banking-model stack (ALM/IRRBB, liquidity, op-risk capital models). INSURANCE / Solvency II (8) is a separate regime — saved to its own folder. "—" / grey (50) = neither regime (energy, buy-side, ESG, tech, general op/conduct risk); still listed. Editorial — re-sort columns A/B freely.</t>
+          <t>Two prudential regimes, filed separately. BANKING (49) in download waves: Wave 1 Tier-1 core (capital, derivatives, credit derivatives, counterparty/collateral); Wave 2 all remaining credit + regulatory (FRTB, stress testing, IFRS 9/CECL, model risk, systemic); Wave 3 rest of the banking-model stack (ALM/IRRBB, liquidity, op-risk capital models). INSURANCE / Solvency II (8) is a separate regime — saved to its own folder. RISK MISC (50) = everything outside both regimes (op/conduct risk, buy-side, tech/AI, energy, ESG), in its own folder. Editorial — re-sort columns A/B freely.</t>
         </is>
       </c>
     </row>

</xml_diff>